<commit_message>
Corrección de la pregunta 19 (4 OK)
</commit_message>
<xml_diff>
--- a/kahoot de itinerarios academicos y profesionales en el entorno sociolaboral actual.xlsx
+++ b/kahoot de itinerarios academicos y profesionales en el entorno sociolaboral actual.xlsx
@@ -961,9 +961,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>339480</xdr:colOff>
+      <xdr:colOff>339120</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>303480</xdr:rowOff>
+      <xdr:rowOff>303120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -973,7 +973,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="908280" y="228960"/>
-          <a:ext cx="312480" cy="312480"/>
+          <a:ext cx="312120" cy="312120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1001,9 +1001,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>339480</xdr:colOff>
+      <xdr:colOff>339120</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>303480</xdr:rowOff>
+      <xdr:rowOff>303120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1013,7 +1013,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="908280" y="228960"/>
-          <a:ext cx="312480" cy="312480"/>
+          <a:ext cx="312120" cy="312120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1041,9 +1041,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1301760</xdr:colOff>
+      <xdr:colOff>1301400</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>417960</xdr:rowOff>
+      <xdr:rowOff>417600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1057,7 +1057,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="927360" y="228960"/>
-          <a:ext cx="1255680" cy="426960"/>
+          <a:ext cx="1255320" cy="426600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2179,7 +2179,7 @@
         <v>20</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>

</xml_diff>